<commit_message>
fix: stabilize whatsapp campaign blast flow
</commit_message>
<xml_diff>
--- a/docs/data/Format Template.xlsx
+++ b/docs/data/Format Template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acer\Desktop\sampah\item\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acer\Desktop\Project\RUST\Tridjaya Manado\docs\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{789A6FA2-A1A9-4853-A60F-F1293AD210B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EB375DE-08F0-4B8D-B0AE-80537ED832B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="16305" xr2:uid="{0986F36E-3325-4F5B-8A54-5856074FD1D1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>No</t>
   </si>
@@ -65,70 +65,13 @@
     <t>anca</t>
   </si>
   <si>
-    <t>+62 812-4445-9180</t>
-  </si>
-  <si>
-    <t>amel</t>
-  </si>
-  <si>
-    <t>+62 838-9529-5471</t>
-  </si>
-  <si>
-    <t>risna</t>
-  </si>
-  <si>
-    <t>+62 853-4040-7005</t>
-  </si>
-  <si>
-    <t>kak</t>
-  </si>
-  <si>
-    <t>+62 823-5340-6614</t>
-  </si>
-  <si>
-    <t>fey</t>
-  </si>
-  <si>
-    <t>+62 821-8731-8485</t>
-  </si>
-  <si>
-    <t>dayo</t>
-  </si>
-  <si>
-    <t>+62 877-6631-1432</t>
-  </si>
-  <si>
-    <t>eyo</t>
-  </si>
-  <si>
-    <t>+62 856-5708-5482</t>
-  </si>
-  <si>
-    <t>yara</t>
-  </si>
-  <si>
-    <t>+62 812-4117-966</t>
-  </si>
-  <si>
-    <t>Magdalena</t>
-  </si>
-  <si>
-    <t>+62 882-0201-29842</t>
-  </si>
-  <si>
-    <t>Mhyra</t>
-  </si>
-  <si>
-    <t>+62 821-4810-3387</t>
-  </si>
-  <si>
-    <t>asky</t>
-  </si>
-  <si>
-    <t>+62 822-9600-3031</t>
-  </si>
-  <si>
-    <t>etan</t>
+    <t>+62 823-3923-5048</t>
+  </si>
+  <si>
+    <t>+62 882-0212-23128</t>
+  </si>
+  <si>
+    <t>yane 2</t>
   </si>
 </sst>
 </file>
@@ -549,10 +492,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -560,10 +503,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="1">
-        <v>82339235048</v>
+        <v>10</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -571,121 +514,61 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
-        <v>5</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>10</v>
-      </c>
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <v>6</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
-        <v>7</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
-        <v>8</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>16</v>
-      </c>
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
-        <v>9</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>18</v>
-      </c>
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
-        <v>10</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>20</v>
-      </c>
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
-        <v>11</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>22</v>
-      </c>
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
-        <v>12</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="1">
-        <v>13</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>26</v>
-      </c>
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
-        <v>14</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>28</v>
-      </c>
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>